<commit_message>
Updated ColorManager palette for higher contrast and readability
</commit_message>
<xml_diff>
--- a/plans/20260726plan.xlsx
+++ b/plans/20260726plan.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -51,8 +51,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00F2F9FF"/>
+        <bgColor rgb="00F2F9FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFBF0"/>
+        <bgColor rgb="00FFFBF0"/>
       </patternFill>
     </fill>
   </fills>
@@ -68,10 +74,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -441,12 +448,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -493,204 +500,844 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="n"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>NEONSAT1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>First Contact</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>TM 확인 / Panel 전개 / TLE update</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>300.0</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
-      <c r="B3" s="2" t="inlineStr"/>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="n"/>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>NEONSAT1</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Health check</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>EPS / AOCS / S-band 상태 점검</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>180.0</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>First Contact</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr"/>
-      <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="n"/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>NEONSAT1</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Configuration check</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Thermal / STX / FCS param 확인</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>180.0</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Health check</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
-      <c r="B5" s="2" t="inlineStr"/>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="n"/>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>NEONSAT1</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>X-band Key update</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>X key update</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>15.0</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>120.0</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Configuration check</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
-      <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="n"/>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>NEONSAT1</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>1차 지상 촬영</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>시나리오 등록 / 이미징 / 다운로드</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>400.0</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>X-band Key update</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
-      <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="n"/>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>NEONSAT1</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>1차 Cal Maneuver</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>시나리오 등록 / Max logging / AOTM 다운</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>15.0</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>BOTH</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>300.0</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>1차 지상 촬영</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
-      <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="n"/>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>NEONSAT1</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2차 Cal Maneuver</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>시나리오 등록 / Max logging / AOTM 다운</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>15.0</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>BOTH</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>300.0</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>1차 Cal Maneuver</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
-      <c r="B9" s="2" t="inlineStr"/>
-      <c r="C9" s="2" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="n"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>NEONSAT1</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>3차 Cal Maneuver</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>시나리오 등록 / Max logging / AOTM 다운</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>15.0</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>BOTH</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>300.0</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>2차 Cal Maneuver</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
-      <c r="B10" s="2" t="inlineStr"/>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="n"/>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>NEONSAT1</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>FCS Parameter Update</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>FCP 업데이트 (STS-Gyro up)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>180.0</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>3차 Cal Maneuver</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
-      <c r="B11" s="2" t="inlineStr"/>
-      <c r="C11" s="2" t="inlineStr"/>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="n"/>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>NEONSAT1</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>1차 별촬영</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>시나리오 등록 / Max logging / AOTM 다운</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>360.0</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>FCS Parameter Update</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
-      <c r="B12" s="2" t="inlineStr"/>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="n"/>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>NEONSAT-1A</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>First Contact</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>TM 확인 / Panel 전개 / TLE update</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>300.0</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
-      <c r="B13" s="2" t="inlineStr"/>
-      <c r="C13" s="2" t="inlineStr"/>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="n"/>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>NEONSAT-1A</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Health check</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>EPS / AOCS / S-band 상태 점검</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>180.0</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>First Contact</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
-      <c r="B14" s="2" t="inlineStr"/>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="n"/>
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>NEONSAT-1A</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Configuration check</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Thermal / STX / FCS param 확인</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>180.0</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Health check</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
-      <c r="B15" s="2" t="inlineStr"/>
-      <c r="C15" s="2" t="inlineStr"/>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr"/>
-      <c r="G15" s="2" t="inlineStr"/>
-      <c r="H15" s="2" t="n"/>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>NEONSAT-1A</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>X-band Key update</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>X key update</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>15.0</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>120.0</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Configuration check</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
-      <c r="B16" s="2" t="inlineStr"/>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr"/>
-      <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="2" t="n"/>
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>NEONSAT-1A</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>1차 지상 촬영</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>시나리오 등록 / 이미징 / 다운로드</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>400.0</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>X-band Key update</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr"/>
-      <c r="B17" s="2" t="inlineStr"/>
-      <c r="C17" s="2" t="inlineStr"/>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr"/>
-      <c r="G17" s="2" t="inlineStr"/>
-      <c r="H17" s="2" t="n"/>
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>NEONSAT-1A</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>1차 Cal Maneuver</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>시나리오 등록 / Max logging / AOTM 다운</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>15.0</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>BOTH</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>300.0</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>1차 지상 촬영</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
-      <c r="B18" s="2" t="inlineStr"/>
-      <c r="C18" s="2" t="inlineStr"/>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr"/>
-      <c r="G18" s="2" t="inlineStr"/>
-      <c r="H18" s="2" t="n"/>
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>NEONSAT-1A</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>2차 Cal Maneuver</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>시나리오 등록 / Max logging / AOTM 다운</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>15.0</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>BOTH</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>300.0</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>1차 Cal Maneuver</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
-      <c r="B19" s="2" t="inlineStr"/>
-      <c r="C19" s="2" t="inlineStr"/>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr"/>
-      <c r="G19" s="2" t="inlineStr"/>
-      <c r="H19" s="2" t="n"/>
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>NEONSAT-1A</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>3차 Cal Maneuver</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>시나리오 등록 / Max logging / AOTM 다운</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>15.0</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>BOTH</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>300.0</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>2차 Cal Maneuver</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
-      <c r="B20" s="2" t="inlineStr"/>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr"/>
-      <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="n"/>
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>NEONSAT-1A</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>FCS Parameter Update</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>FCP 업데이트 (STS-Gyro up)</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>180.0</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>3차 Cal Maneuver</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr"/>
-      <c r="B21" s="2" t="inlineStr"/>
-      <c r="C21" s="2" t="inlineStr"/>
-      <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="2" t="inlineStr"/>
-      <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="2" t="inlineStr"/>
-      <c r="H21" s="2" t="n"/>
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>NEONSAT-1A</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>1차 별촬영</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>시나리오 등록 / Max logging / AOTM 다운</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>360.0</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>FCS Parameter Update</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>